<commit_message>
Revue qualité : 8.11 réintégrée (cohérence avec 8.33), traçabilité risques/actions, articles 09-08 et décret 2-21-406 vérifiés, coût A17 réaliste, corrections LEARN
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/gap_analysis_annexA.xlsx
+++ b/outputs/gap_analysis_annexA.xlsx
@@ -4610,7 +4610,7 @@
       </c>
       <c r="M68" s="2" t="inlineStr">
         <is>
-          <t>R03, R08</t>
+          <t>R02, R03, R08</t>
         </is>
       </c>
     </row>
@@ -4764,40 +4764,38 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Pas d'environnement de test contenant des données réelles à ce jour.</t>
-        </is>
-      </c>
-      <c r="H71" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I71" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="J71" s="2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+          <t>Tests occasionnels avec de vraies commandes clients (voir 8.33) ; exports complets du fichier transmis au transporteur sans réduction des champs.</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I71" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J71" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>Non applicable à ce stade.</t>
+          <t>Pseudonymiser/anonymiser les données utilisées hors production et les anciennes commandes (lien 8.10, 8.33) ; exports transporteur limités au strict nécessaire.</t>
         </is>
       </c>
       <c r="L71" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M71" s="2" t="inlineStr"/>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>R03, R09</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -5584,7 +5582,7 @@
       </c>
       <c r="M84" s="2" t="inlineStr">
         <is>
-          <t>R03, R12</t>
+          <t>R03, R04, R12</t>
         </is>
       </c>
     </row>
@@ -8261,7 +8259,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Traitement des risques R03, R08</t>
+          <t>Traitement des risques R02, R03, R08</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -8352,20 +8350,24 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Non</t>
+          <t>Oui</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Exclue provisoirement : aucune copie de données de production hors production. À réintégrer si une préproduction est créée (action A21) - lien avec 8.33.</t>
+          <t>Traitement des risques R03, R09 ; minimisation (loi 09-08, art. 3). Exclusion initialement envisagée puis écartée : des données réelles sont utilisées en test (8.33).</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Non applicable</t>
-        </is>
-      </c>
-      <c r="F71" s="2" t="inlineStr"/>
+          <t>Non mis en oeuvre</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>A15</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -8745,7 +8747,7 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Traitement des risques R03, R12</t>
+          <t>Traitement des risques R03, R04, R12</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -9179,13 +9181,13 @@
         <v>34</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.73</v>
+        <v>0.71</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>2.3</v>
+        <v>2.29</v>
       </c>
     </row>
     <row r="6">
@@ -9356,7 +9358,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>A01, A03, A12, A19</t>
+          <t>A01, A03, A12, A16, A18, A19</t>
         </is>
       </c>
       <c r="K2" s="2" t="n">
@@ -9416,7 +9418,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>A04, A09, A12, A20</t>
+          <t>A04, A09, A12, A16, A20</t>
         </is>
       </c>
       <c r="K3" s="2" t="n">
@@ -9476,7 +9478,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>A05, A17, A21</t>
+          <t>A05, A16, A17, A18, A21, A23</t>
         </is>
       </c>
       <c r="K4" s="2" t="n">
@@ -9596,7 +9598,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>A01, A03, A08</t>
+          <t>A01, A03, A08, A18</t>
         </is>
       </c>
       <c r="K6" s="2" t="n">
@@ -9776,7 +9778,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>A05, A17, A23</t>
+          <t>A05, A17, A21, A23</t>
         </is>
       </c>
       <c r="K9" s="2" t="n">
@@ -9831,12 +9833,12 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>5.31, 5.34, 5.20, 8.10</t>
+          <t>5.20, 5.31, 5.34, 8.10, 8.11</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>A10, A13, A14, A15</t>
+          <t>A10, A13, A14, A15, A19</t>
         </is>
       </c>
       <c r="K10" s="2" t="n">
@@ -9956,7 +9958,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>A08, A11, A14</t>
+          <t>A08, A11, A14, A19</t>
         </is>
       </c>
       <c r="K12" s="2" t="n">
@@ -10727,7 +10729,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>5.9, 5.12, 8.10</t>
+          <t>5.9, 5.12, 8.10, 8.11</t>
         </is>
       </c>
     </row>
@@ -10796,7 +10798,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>10 000 - 25 000</t>
+          <t>25 000 - 50 000</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">

</xml_diff>